<commit_message>
Sync desktop project and update website
Sync desktop project and update website
</commit_message>
<xml_diff>
--- a/reports/TSLA_Simon_Valuation.xlsx
+++ b/reports/TSLA_Simon_Valuation.xlsx
@@ -11,6 +11,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical FCFE" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF Audit" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peer Multiples" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comps Valuation" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analyst Consensus" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,10 +23,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="0.00x"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,6 +48,9 @@
     <font>
       <b val="1"/>
       <i val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -70,7 +78,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -78,6 +86,8 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -542,8 +552,9 @@
           <t>Cost of common equity (Ke)</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n">
-        <v>0.138615</v>
+      <c r="B10" s="2">
+        <f>B7+B9*B8</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -583,7 +594,7 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>5427500000</v>
+        <v>6220000000</v>
       </c>
     </row>
     <row r="15">
@@ -603,7 +614,7 @@
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>420.11</v>
+        <v>415.88</v>
       </c>
     </row>
     <row r="17">
@@ -613,7 +624,7 @@
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>15.33371967889497</v>
+        <v>17.57268289317858</v>
       </c>
     </row>
   </sheetData>
@@ -823,7 +834,7 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>5427500000</v>
+        <v>6220000000</v>
       </c>
     </row>
   </sheetData>
@@ -1015,7 +1026,7 @@
       </c>
       <c r="G19" s="3" t="n"/>
       <c r="H19" s="3" t="n">
-        <v>5563187499.999999</v>
+        <v>6375499999.999999</v>
       </c>
     </row>
     <row r="20">
@@ -1034,7 +1045,7 @@
       <c r="F20" s="3" t="n"/>
       <c r="G20" s="3" t="n"/>
       <c r="H20" s="3" t="n">
-        <v>5702267187.499998</v>
+        <v>6534887499.999998</v>
       </c>
     </row>
     <row r="21">
@@ -1053,7 +1064,7 @@
       <c r="F21" s="3" t="n"/>
       <c r="G21" s="3" t="n"/>
       <c r="H21" s="3" t="n">
-        <v>5844823867.187497</v>
+        <v>6698259687.499997</v>
       </c>
       <c r="I21" s="2">
         <f>Assumptions!B11</f>
@@ -1076,7 +1087,7 @@
       <c r="F22" s="3" t="n"/>
       <c r="G22" s="3" t="n"/>
       <c r="H22" s="3" t="n">
-        <v>5990944463.867184</v>
+        <v>6865716179.687496</v>
       </c>
     </row>
     <row r="23">
@@ -1095,7 +1106,7 @@
       <c r="F23" s="3" t="n"/>
       <c r="G23" s="3" t="n"/>
       <c r="H23" s="3" t="n">
-        <v>6140718075.463862</v>
+        <v>7037359084.179683</v>
       </c>
     </row>
     <row r="24">
@@ -1134,7 +1145,7 @@
       <c r="F26" s="3" t="n"/>
       <c r="G26" s="3" t="n"/>
       <c r="H26" s="3" t="n">
-        <v>57589217029.24828</v>
+        <v>65998144619.42413</v>
       </c>
     </row>
     <row r="27">
@@ -1164,7 +1175,7 @@
       <c r="F28" s="4" t="n"/>
       <c r="G28" s="4" t="n"/>
       <c r="H28" s="4" t="n">
-        <v>15.33371967889497</v>
+        <v>17.57268289317858</v>
       </c>
     </row>
   </sheetData>
@@ -1281,7 +1292,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>$5.43B</t>
+          <t>$6.22B</t>
         </is>
       </c>
     </row>
@@ -1309,7 +1320,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>$5.56B</t>
+          <t>$6.38B</t>
         </is>
       </c>
     </row>
@@ -1321,7 +1332,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>$5.70B</t>
+          <t>$6.53B</t>
         </is>
       </c>
     </row>
@@ -1333,7 +1344,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>$5.84B</t>
+          <t>$6.70B</t>
         </is>
       </c>
     </row>
@@ -1345,7 +1356,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>$5.99B</t>
+          <t>$6.87B</t>
         </is>
       </c>
     </row>
@@ -1357,7 +1368,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$6.14B</t>
+          <t>$7.04B</t>
         </is>
       </c>
     </row>
@@ -1381,7 +1392,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>$6.39B</t>
+          <t>$7.32B</t>
         </is>
       </c>
     </row>
@@ -1393,7 +1404,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>$64.76B</t>
+          <t>$74.22B</t>
         </is>
       </c>
     </row>
@@ -1413,7 +1424,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>$53.86B</t>
+          <t>$61.72B</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1448,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>$57.59B</t>
+          <t>$66.00B</t>
         </is>
       </c>
     </row>
@@ -1461,7 +1472,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>$15.33</t>
+          <t>$17.57</t>
         </is>
       </c>
     </row>
@@ -1473,8 +1484,717 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>-96.4%</t>
-        </is>
+          <t>-95.8%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Comparable company multiples (Yahoo Finance)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>P/E and EV/EBITDA medians include subject; P/S median uses peers only (matches Python model).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>P/E</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>EV/EBITDA</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>P/S</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ford Motor Company</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="n"/>
+      <c r="D5" s="7" t="n">
+        <v>27.35</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>0.34902078</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>GM</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>General Motors Company</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>30.175182</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>9.920999999999999</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>0.4037941</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>RIVN</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Rivian Automotive, Inc.</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="n"/>
+      <c r="D7" s="7" t="n">
+        <v>-6.915</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>4.1175084</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TM</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Toyota Motor Corporation</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>9.887567499999999</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>5.325</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>0.004703697</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>381.5413</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>144.992</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>15.957768</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Median P/E (peers + subject)</t>
+        </is>
+      </c>
+      <c r="C10">
+        <f>MEDIAN(C5:C9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Median EV/EBITDA (peers + subject)</t>
+        </is>
+      </c>
+      <c r="D11">
+        <f>MEDIAN(D5:D9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Median P/S (peers only)</t>
+        </is>
+      </c>
+      <c r="E12">
+        <f>MEDIAN(E5:E8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Python reference (peer_median_pe)</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>30.175182</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Python reference (peer_median_ev_ebitda)</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>9.920999999999999</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Python reference (peer_median_ps)</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>0.4037941</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Comparable multiples — implied share price</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Implied price = f(peer median multiple, subject fundamentals, shares outstanding).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Subject fundamentals</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Trailing EPS ($/sh)</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>1.09</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>EBITDA ($)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>11764000000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Revenue ($)</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>94827000000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Net debt ($)</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>-1794000000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Shares outstanding</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>3755723871</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Current price ($/sh)</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>415.88</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Calculation (formula)</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Implied $/sh</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>P/E (peer median × EPS)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Median P/E × B5 (EPS)</t>
+        </is>
+      </c>
+      <c r="C13" s="4">
+        <f>IF(OR('Peer Multiples'!C10="",B5="",B5&lt;=0),"",'Peer Multiples'!C10*B5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>EV/EBITDA (implied equity / shares)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>(Median EV/EBITDA × B6 − B8) / B9</t>
+        </is>
+      </c>
+      <c r="C14" s="4">
+        <f>IF(OR('Peer Multiples'!D11="",B6="",B6&lt;=0,B9="",B9&lt;=0),"",(('Peer Multiples'!D11*B6)-B8)/B9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>P/S (implied equity / shares)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>(Median P/S × B7) / B9</t>
+        </is>
+      </c>
+      <c r="C15" s="4">
+        <f>IF(OR('Peer Multiples'!E12="",B7="",B7&lt;=0,B9="",B9&lt;=0),"",('Peer Multiples'!E12*B7)/B9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Comps blended (average of available)</t>
+        </is>
+      </c>
+      <c r="B16">
+        <f>AVERAGE(C13:C15)</f>
+        <v/>
+      </c>
+      <c r="C16" s="4">
+        <f>IF(COUNT(C13,C14,C15)=0,"",AVERAGE(C13,C14,C15))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Python reference (blended_fair_value)</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>24.87976190651591</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Analyst consensus (Yahoo Finance targetMeanPrice)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Used as one input to the blended target (no formula derivation — market consensus).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Analyst mean target ($/sh)</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>411.8878</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Current price ($/sh)</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>415.88</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Upside vs. current</t>
+        </is>
+      </c>
+      <c r="B7" s="2">
+        <f>IF(OR(B5="",B6="",B6=0),"",B5/B6-1)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Multi-method valuation — blended target</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Base weights: DCF 28%, Comps 44%, Analyst 28%. Effective weights reflect outlier / reliability exclusions from the Python model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Implied $/sh</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>vs. Current</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Base weight</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Effective weight</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DCF (Simon FCFE)</t>
+        </is>
+      </c>
+      <c r="B5" s="4">
+        <f>DCF!B28</f>
+        <v/>
+      </c>
+      <c r="C5" s="2">
+        <f>IF(OR(B5="",'Comps Valuation'!B10="",'Comps Valuation'!B10=0),"",B5/'Comps Valuation'!B10-1)</f>
+        <v/>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>DCF implied price &lt; 35% of market (capex-heavy or distorted FCFE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Comps (blended multiples)</t>
+        </is>
+      </c>
+      <c r="B6" s="4">
+        <f>'Comps Valuation'!C16</f>
+        <v/>
+      </c>
+      <c r="C6" s="2">
+        <f>IF(OR(B6="",'Comps Valuation'!B10="",'Comps Valuation'!B10=0),"",B6/'Comps Valuation'!B10-1)</f>
+        <v/>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Diverges below other methods (6% of median)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Analyst consensus</t>
+        </is>
+      </c>
+      <c r="B7" s="4">
+        <f>'Analyst Consensus'!B5</f>
+        <v/>
+      </c>
+      <c r="C7" s="2">
+        <f>IF(OR(B7="",'Comps Valuation'!B10="",'Comps Valuation'!B10=0),"",B7/'Comps Valuation'!B10-1)</f>
+        <v/>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Included in blend</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Blended target (effective weights)</t>
+        </is>
+      </c>
+      <c r="B9" s="4">
+        <f>SUMPRODUCT(E5:E7,B5:B7)</f>
+        <v/>
+      </c>
+      <c r="C9" s="2">
+        <f>IF(OR(B9="",'Comps Valuation'!B10="",'Comps Valuation'!B10=0),"",B9/'Comps Valuation'!B10-1)</f>
+        <v/>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>HOLD - Fairly valued</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Formula check (if all methods included, normalized base weights)</t>
+        </is>
+      </c>
+      <c r="B11" s="4">
+        <f>SUMPRODUCT($D$5:$D$7/SUM($D$5:$D$7),B5:B7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Python reference (target_price)</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>411.8878</v>
       </c>
     </row>
   </sheetData>

</xml_diff>